<commit_message>
colocar unidades de medidas que se usan en Venezuela
</commit_message>
<xml_diff>
--- a/public/formats/items.xlsx
+++ b/public/formats/items.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" r:id="Ra7855a48804043ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" r:id="R55828699b0db491c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,9 +65,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">GA001</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NIU</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">NO</x:t>
@@ -406,8 +403,8 @@
       <x:c r="D2">
         <x:v>51121703</x:v>
       </x:c>
-      <x:c r="E2" t="s">
-        <x:v>19</x:v>
+      <x:c r="E2" t="str">
+        <x:v>UND</x:v>
       </x:c>
       <x:c r="F2" t="str">
         <x:v>VES</x:v>
@@ -419,7 +416,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="I2" t="s">
-        <x:v>20</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="J2">
         <x:v>70</x:v>
@@ -434,10 +431,10 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="N2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="O2" t="s">
         <x:v>21</x:v>
-      </x:c>
-      <x:c r="O2" t="s">
-        <x:v>22</x:v>
       </x:c>
       <x:c r="P2" t="s">
         <x:v>16</x:v>
@@ -447,7 +444,7 @@
       </x:c>
       <x:c r="S2" s="1"/>
       <x:c r="T2" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>